<commit_message>
Updated trade execution logic and added back of queue model
</commit_message>
<xml_diff>
--- a/sheets/quote_position.xlsx
+++ b/sheets/quote_position.xlsx
@@ -1,17 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AAPL" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AMZN" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GE" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IVV" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="AAPL" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="AAPL_back" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="AMZN" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="AMZN_back" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="GE" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="GE_back" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="IVV" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="IVV_back" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="M" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="M_back" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -423,7 +428,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Day 1 — Active seconds: 10864</t>
+          <t>Day 1 — Active seconds: 13013</t>
         </is>
       </c>
     </row>
@@ -456,13 +461,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1066</v>
+        <v>1788</v>
       </c>
       <c r="C3" t="n">
-        <v>1764</v>
+        <v>2104</v>
       </c>
       <c r="D3" t="n">
-        <v>8034</v>
+        <v>9121</v>
       </c>
     </row>
     <row r="4">
@@ -472,13 +477,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>371</v>
+        <v>1199</v>
       </c>
       <c r="C4" t="n">
-        <v>956</v>
+        <v>1531</v>
       </c>
       <c r="D4" t="n">
-        <v>2386</v>
+        <v>4041</v>
       </c>
     </row>
     <row r="6">
@@ -510,13 +515,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>9.800000000000001</v>
+        <v>13.7</v>
       </c>
       <c r="C7" t="n">
         <v>16.2</v>
       </c>
       <c r="D7" t="n">
-        <v>74</v>
+        <v>70.09999999999999</v>
       </c>
     </row>
     <row r="8">
@@ -526,19 +531,19 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>3.4</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="C8" t="n">
-        <v>8.800000000000001</v>
+        <v>11.8</v>
       </c>
       <c r="D8" t="n">
-        <v>22</v>
+        <v>31.1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Day 2 — Active seconds: 14235</t>
+          <t>Day 2 — Active seconds: 15868</t>
         </is>
       </c>
     </row>
@@ -571,13 +576,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1042</v>
+        <v>1508</v>
       </c>
       <c r="C13" t="n">
-        <v>2566</v>
+        <v>2900</v>
       </c>
       <c r="D13" t="n">
-        <v>10627</v>
+        <v>11460</v>
       </c>
     </row>
     <row r="14">
@@ -587,13 +592,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>515</v>
+        <v>1205</v>
       </c>
       <c r="C14" t="n">
-        <v>1853</v>
+        <v>2473</v>
       </c>
       <c r="D14" t="n">
-        <v>4852</v>
+        <v>7061</v>
       </c>
     </row>
     <row r="16">
@@ -625,13 +630,13 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>7.3</v>
+        <v>9.5</v>
       </c>
       <c r="C17" t="n">
-        <v>18</v>
+        <v>18.3</v>
       </c>
       <c r="D17" t="n">
-        <v>74.7</v>
+        <v>72.2</v>
       </c>
     </row>
     <row r="18">
@@ -641,19 +646,19 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>3.6</v>
+        <v>7.6</v>
       </c>
       <c r="C18" t="n">
-        <v>13</v>
+        <v>15.6</v>
       </c>
       <c r="D18" t="n">
-        <v>34.1</v>
+        <v>44.5</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Day 3 — Active seconds: 13239</t>
+          <t>Day 3 — Active seconds: 15422</t>
         </is>
       </c>
     </row>
@@ -686,13 +691,13 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1178</v>
+        <v>1864</v>
       </c>
       <c r="C23" t="n">
-        <v>1691</v>
+        <v>1932</v>
       </c>
       <c r="D23" t="n">
-        <v>10370</v>
+        <v>11626</v>
       </c>
     </row>
     <row r="24">
@@ -702,13 +707,13 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>564</v>
+        <v>1352</v>
       </c>
       <c r="C24" t="n">
-        <v>1020</v>
+        <v>1479</v>
       </c>
       <c r="D24" t="n">
-        <v>4976</v>
+        <v>7149</v>
       </c>
     </row>
     <row r="26">
@@ -740,13 +745,13 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>8.9</v>
+        <v>12.1</v>
       </c>
       <c r="C27" t="n">
-        <v>12.8</v>
+        <v>12.5</v>
       </c>
       <c r="D27" t="n">
-        <v>78.3</v>
+        <v>75.40000000000001</v>
       </c>
     </row>
     <row r="28">
@@ -756,19 +761,19 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>4.3</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="C28" t="n">
-        <v>7.7</v>
+        <v>9.6</v>
       </c>
       <c r="D28" t="n">
-        <v>37.6</v>
+        <v>46.4</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Day 4 — Active seconds: 14184</t>
+          <t>Day 4 — Active seconds: 15957</t>
         </is>
       </c>
     </row>
@@ -801,13 +806,13 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>803</v>
+        <v>1366</v>
       </c>
       <c r="C33" t="n">
-        <v>2159</v>
+        <v>2581</v>
       </c>
       <c r="D33" t="n">
-        <v>11222</v>
+        <v>12010</v>
       </c>
     </row>
     <row r="34">
@@ -817,13 +822,13 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>464</v>
+        <v>1087</v>
       </c>
       <c r="C34" t="n">
-        <v>1459</v>
+        <v>2182</v>
       </c>
       <c r="D34" t="n">
-        <v>5256</v>
+        <v>7400</v>
       </c>
     </row>
     <row r="36">
@@ -855,13 +860,13 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>5.7</v>
+        <v>8.6</v>
       </c>
       <c r="C37" t="n">
-        <v>15.2</v>
+        <v>16.2</v>
       </c>
       <c r="D37" t="n">
-        <v>79.09999999999999</v>
+        <v>75.3</v>
       </c>
     </row>
     <row r="38">
@@ -871,19 +876,19 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>3.3</v>
+        <v>6.8</v>
       </c>
       <c r="C38" t="n">
-        <v>10.3</v>
+        <v>13.7</v>
       </c>
       <c r="D38" t="n">
-        <v>37.1</v>
+        <v>46.4</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Day 5 — Active seconds: 14893</t>
+          <t>Day 5 — Active seconds: 16699</t>
         </is>
       </c>
     </row>
@@ -916,13 +921,13 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>757</v>
+        <v>1196</v>
       </c>
       <c r="C43" t="n">
-        <v>2310</v>
+        <v>2669</v>
       </c>
       <c r="D43" t="n">
-        <v>11826</v>
+        <v>12834</v>
       </c>
     </row>
     <row r="44">
@@ -932,13 +937,13 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>476</v>
+        <v>1015</v>
       </c>
       <c r="C44" t="n">
-        <v>1740</v>
+        <v>2249</v>
       </c>
       <c r="D44" t="n">
-        <v>5939</v>
+        <v>8213</v>
       </c>
     </row>
     <row r="46">
@@ -970,13 +975,13 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>5.1</v>
+        <v>7.2</v>
       </c>
       <c r="C47" t="n">
-        <v>15.5</v>
+        <v>16</v>
       </c>
       <c r="D47" t="n">
-        <v>79.40000000000001</v>
+        <v>76.90000000000001</v>
       </c>
     </row>
     <row r="48">
@@ -986,13 +991,602 @@
         </is>
       </c>
       <c r="B48" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="C48" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="D48" t="n">
+        <v>49.2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D48"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Day 1 — Active seconds: 18175</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Counts</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Inside NBBO</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>At NBBO</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Outside NBBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>814</v>
+      </c>
+      <c r="C3" t="n">
+        <v>15665</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1696</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>529</v>
+      </c>
+      <c r="C4" t="n">
+        <v>13372</v>
+      </c>
+      <c r="D4" t="n">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Percentages (%)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Inside NBBO</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>At NBBO</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Outside NBBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="C7" t="n">
+        <v>86.2</v>
+      </c>
+      <c r="D7" t="n">
+        <v>9.300000000000001</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="C8" t="n">
+        <v>73.59999999999999</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Day 2 — Active seconds: 18250</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Counts</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Inside NBBO</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>At NBBO</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Outside NBBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>220</v>
+      </c>
+      <c r="C13" t="n">
+        <v>16922</v>
+      </c>
+      <c r="D13" t="n">
+        <v>1108</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>153</v>
+      </c>
+      <c r="C14" t="n">
+        <v>15429</v>
+      </c>
+      <c r="D14" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Percentages (%)</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Inside NBBO</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>At NBBO</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Outside NBBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="C17" t="n">
+        <v>92.7</v>
+      </c>
+      <c r="D17" t="n">
+        <v>6.1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="C18" t="n">
+        <v>84.5</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Day 3 — Active seconds: 19224</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Counts</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Inside NBBO</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>At NBBO</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Outside NBBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>619</v>
+      </c>
+      <c r="C23" t="n">
+        <v>17319</v>
+      </c>
+      <c r="D23" t="n">
+        <v>1286</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>463</v>
+      </c>
+      <c r="C24" t="n">
+        <v>15519</v>
+      </c>
+      <c r="D24" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Percentages (%)</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Inside NBBO</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>At NBBO</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Outside NBBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
         <v>3.2</v>
       </c>
+      <c r="C27" t="n">
+        <v>90.09999999999999</v>
+      </c>
+      <c r="D27" t="n">
+        <v>6.7</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="C28" t="n">
+        <v>80.7</v>
+      </c>
+      <c r="D28" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Day 4 — Active seconds: 19386</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Counts</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Inside NBBO</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>At NBBO</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Outside NBBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>515</v>
+      </c>
+      <c r="C33" t="n">
+        <v>17888</v>
+      </c>
+      <c r="D33" t="n">
+        <v>983</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>338</v>
+      </c>
+      <c r="C34" t="n">
+        <v>16135</v>
+      </c>
+      <c r="D34" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Percentages (%)</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Inside NBBO</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>At NBBO</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Outside NBBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="C37" t="n">
+        <v>92.3</v>
+      </c>
+      <c r="D37" t="n">
+        <v>5.1</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="C38" t="n">
+        <v>83.2</v>
+      </c>
+      <c r="D38" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Day 5 — Active seconds: 19624</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Counts</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Inside NBBO</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>At NBBO</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Outside NBBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>561</v>
+      </c>
+      <c r="C43" t="n">
+        <v>17896</v>
+      </c>
+      <c r="D43" t="n">
+        <v>1167</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>377</v>
+      </c>
+      <c r="C44" t="n">
+        <v>15750</v>
+      </c>
+      <c r="D44" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Percentages (%)</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Inside NBBO</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>At NBBO</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Outside NBBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="C47" t="n">
+        <v>91.2</v>
+      </c>
+      <c r="D47" t="n">
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>1.9</v>
+      </c>
       <c r="C48" t="n">
-        <v>11.7</v>
+        <v>80.3</v>
       </c>
       <c r="D48" t="n">
-        <v>39.9</v>
+        <v>0.2</v>
       </c>
     </row>
   </sheetData>
@@ -1012,7 +1606,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Day 1 — Active seconds: 13983</t>
+          <t>Day 1 — Active seconds: 18090</t>
         </is>
       </c>
     </row>
@@ -1045,13 +1639,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>5921</v>
+        <v>3663</v>
       </c>
       <c r="C3" t="n">
-        <v>114</v>
+        <v>3436</v>
       </c>
       <c r="D3" t="n">
-        <v>7948</v>
+        <v>10991</v>
       </c>
     </row>
     <row r="4">
@@ -1061,13 +1655,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2476</v>
+        <v>3001</v>
       </c>
       <c r="C4" t="n">
-        <v>59</v>
+        <v>3277</v>
       </c>
       <c r="D4" t="n">
-        <v>4579</v>
+        <v>8975</v>
       </c>
     </row>
     <row r="6">
@@ -1099,13 +1693,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>42.3</v>
+        <v>20.2</v>
       </c>
       <c r="C7" t="n">
-        <v>0.8</v>
+        <v>19</v>
       </c>
       <c r="D7" t="n">
-        <v>56.8</v>
+        <v>60.8</v>
       </c>
     </row>
     <row r="8">
@@ -1115,19 +1709,19 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>17.7</v>
+        <v>16.6</v>
       </c>
       <c r="C8" t="n">
-        <v>0.4</v>
+        <v>18.1</v>
       </c>
       <c r="D8" t="n">
-        <v>32.7</v>
+        <v>49.6</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Day 2 — Active seconds: 17795</t>
+          <t>Day 2 — Active seconds: 21108</t>
         </is>
       </c>
     </row>
@@ -1160,13 +1754,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>5245</v>
+        <v>2990</v>
       </c>
       <c r="C13" t="n">
-        <v>103</v>
+        <v>4575</v>
       </c>
       <c r="D13" t="n">
-        <v>12447</v>
+        <v>13543</v>
       </c>
     </row>
     <row r="14">
@@ -1176,13 +1770,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>2678</v>
+        <v>2629</v>
       </c>
       <c r="C14" t="n">
-        <v>69</v>
+        <v>4368</v>
       </c>
       <c r="D14" t="n">
-        <v>9171</v>
+        <v>12660</v>
       </c>
     </row>
     <row r="16">
@@ -1214,13 +1808,13 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>29.5</v>
+        <v>14.2</v>
       </c>
       <c r="C17" t="n">
-        <v>0.6</v>
+        <v>21.7</v>
       </c>
       <c r="D17" t="n">
-        <v>69.90000000000001</v>
+        <v>64.2</v>
       </c>
     </row>
     <row r="18">
@@ -1230,19 +1824,19 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>15</v>
+        <v>12.5</v>
       </c>
       <c r="C18" t="n">
-        <v>0.4</v>
+        <v>20.7</v>
       </c>
       <c r="D18" t="n">
-        <v>51.5</v>
+        <v>60</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Day 3 — Active seconds: 17546</t>
+          <t>Day 3 — Active seconds: 20458</t>
         </is>
       </c>
     </row>
@@ -1275,13 +1869,13 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>4807</v>
+        <v>3362</v>
       </c>
       <c r="C23" t="n">
-        <v>218</v>
+        <v>3535</v>
       </c>
       <c r="D23" t="n">
-        <v>12521</v>
+        <v>13561</v>
       </c>
     </row>
     <row r="24">
@@ -1291,13 +1885,13 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>2537</v>
+        <v>2904</v>
       </c>
       <c r="C24" t="n">
-        <v>121</v>
+        <v>3448</v>
       </c>
       <c r="D24" t="n">
-        <v>10287</v>
+        <v>12290</v>
       </c>
     </row>
     <row r="26">
@@ -1329,13 +1923,13 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>27.4</v>
+        <v>16.4</v>
       </c>
       <c r="C27" t="n">
-        <v>1.2</v>
+        <v>17.3</v>
       </c>
       <c r="D27" t="n">
-        <v>71.40000000000001</v>
+        <v>66.3</v>
       </c>
     </row>
     <row r="28">
@@ -1345,19 +1939,19 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>14.5</v>
+        <v>14.2</v>
       </c>
       <c r="C28" t="n">
-        <v>0.7</v>
+        <v>16.9</v>
       </c>
       <c r="D28" t="n">
-        <v>58.6</v>
+        <v>60.1</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Day 4 — Active seconds: 17030</t>
+          <t>Day 4 — Active seconds: 21521</t>
         </is>
       </c>
     </row>
@@ -1390,13 +1984,13 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>4591</v>
+        <v>2716</v>
       </c>
       <c r="C33" t="n">
-        <v>146</v>
+        <v>4169</v>
       </c>
       <c r="D33" t="n">
-        <v>12293</v>
+        <v>14636</v>
       </c>
     </row>
     <row r="34">
@@ -1406,13 +2000,13 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>2334</v>
+        <v>2488</v>
       </c>
       <c r="C34" t="n">
-        <v>78</v>
+        <v>4038</v>
       </c>
       <c r="D34" t="n">
-        <v>9106</v>
+        <v>13776</v>
       </c>
     </row>
     <row r="36">
@@ -1444,13 +2038,13 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>27</v>
+        <v>12.6</v>
       </c>
       <c r="C37" t="n">
-        <v>0.9</v>
+        <v>19.4</v>
       </c>
       <c r="D37" t="n">
-        <v>72.2</v>
+        <v>68</v>
       </c>
     </row>
     <row r="38">
@@ -1460,19 +2054,19 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>13.7</v>
+        <v>11.6</v>
       </c>
       <c r="C38" t="n">
-        <v>0.5</v>
+        <v>18.8</v>
       </c>
       <c r="D38" t="n">
-        <v>53.5</v>
+        <v>64</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Day 5 — Active seconds: 16793</t>
+          <t>Day 5 — Active seconds: 22067</t>
         </is>
       </c>
     </row>
@@ -1505,13 +2099,13 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>1871</v>
+        <v>2469</v>
       </c>
       <c r="C43" t="n">
-        <v>60</v>
+        <v>4216</v>
       </c>
       <c r="D43" t="n">
-        <v>14862</v>
+        <v>15382</v>
       </c>
     </row>
     <row r="44">
@@ -1521,13 +2115,13 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>837</v>
+        <v>2426</v>
       </c>
       <c r="C44" t="n">
-        <v>30</v>
+        <v>4100</v>
       </c>
       <c r="D44" t="n">
-        <v>10839</v>
+        <v>14577</v>
       </c>
     </row>
     <row r="46">
@@ -1559,13 +2153,13 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>11.1</v>
+        <v>11.2</v>
       </c>
       <c r="C47" t="n">
-        <v>0.4</v>
+        <v>19.1</v>
       </c>
       <c r="D47" t="n">
-        <v>88.5</v>
+        <v>69.7</v>
       </c>
     </row>
     <row r="48">
@@ -1575,13 +2169,13 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="C48" t="n">
-        <v>0.2</v>
+        <v>18.6</v>
       </c>
       <c r="D48" t="n">
-        <v>64.5</v>
+        <v>66.09999999999999</v>
       </c>
     </row>
   </sheetData>
@@ -1601,7 +2195,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Day 1 — Active seconds: 12803</t>
+          <t>Day 1 — Active seconds: 17831</t>
         </is>
       </c>
     </row>
@@ -1634,13 +2228,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>14</v>
+        <v>8734</v>
       </c>
       <c r="C3" t="n">
-        <v>11878</v>
+        <v>170</v>
       </c>
       <c r="D3" t="n">
-        <v>911</v>
+        <v>8927</v>
       </c>
     </row>
     <row r="4">
@@ -1650,13 +2244,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>7272</v>
       </c>
       <c r="C4" t="n">
-        <v>3182</v>
+        <v>116</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>6710</v>
       </c>
     </row>
     <row r="6">
@@ -1688,13 +2282,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.1</v>
+        <v>49</v>
       </c>
       <c r="C7" t="n">
-        <v>92.8</v>
+        <v>1</v>
       </c>
       <c r="D7" t="n">
-        <v>7.1</v>
+        <v>50.1</v>
       </c>
     </row>
     <row r="8">
@@ -1704,19 +2298,19 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>40.8</v>
       </c>
       <c r="C8" t="n">
-        <v>24.9</v>
+        <v>0.7</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>37.6</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Day 2 — Active seconds: 12988</t>
+          <t>Day 2 — Active seconds: 20674</t>
         </is>
       </c>
     </row>
@@ -1749,13 +2343,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>5</v>
+        <v>6833</v>
       </c>
       <c r="C13" t="n">
-        <v>12566</v>
+        <v>166</v>
       </c>
       <c r="D13" t="n">
-        <v>417</v>
+        <v>13675</v>
       </c>
     </row>
     <row r="14">
@@ -1765,13 +2359,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>3</v>
+        <v>6303</v>
       </c>
       <c r="C14" t="n">
-        <v>5305</v>
+        <v>117</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>12149</v>
       </c>
     </row>
     <row r="16">
@@ -1803,13 +2397,13 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0</v>
+        <v>33.1</v>
       </c>
       <c r="C17" t="n">
-        <v>96.8</v>
+        <v>0.8</v>
       </c>
       <c r="D17" t="n">
-        <v>3.2</v>
+        <v>66.09999999999999</v>
       </c>
     </row>
     <row r="18">
@@ -1819,19 +2413,19 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0</v>
+        <v>30.5</v>
       </c>
       <c r="C18" t="n">
-        <v>40.8</v>
+        <v>0.6</v>
       </c>
       <c r="D18" t="n">
-        <v>0</v>
+        <v>58.8</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Day 3 — Active seconds: 14425</t>
+          <t>Day 3 — Active seconds: 20407</t>
         </is>
       </c>
     </row>
@@ -1864,13 +2458,13 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>4</v>
+        <v>6561</v>
       </c>
       <c r="C23" t="n">
-        <v>13603</v>
+        <v>134</v>
       </c>
       <c r="D23" t="n">
-        <v>818</v>
+        <v>13712</v>
       </c>
     </row>
     <row r="24">
@@ -1880,13 +2474,13 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>4</v>
+        <v>5729</v>
       </c>
       <c r="C24" t="n">
-        <v>5321</v>
+        <v>188</v>
       </c>
       <c r="D24" t="n">
-        <v>0</v>
+        <v>12504</v>
       </c>
     </row>
     <row r="26">
@@ -1918,13 +2512,13 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>0</v>
+        <v>32.2</v>
       </c>
       <c r="C27" t="n">
-        <v>94.3</v>
+        <v>0.7</v>
       </c>
       <c r="D27" t="n">
-        <v>5.7</v>
+        <v>67.2</v>
       </c>
     </row>
     <row r="28">
@@ -1934,19 +2528,19 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>0</v>
+        <v>28.1</v>
       </c>
       <c r="C28" t="n">
-        <v>36.9</v>
+        <v>0.9</v>
       </c>
       <c r="D28" t="n">
-        <v>0</v>
+        <v>61.3</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Day 4 — Active seconds: 14281</t>
+          <t>Day 4 — Active seconds: 20424</t>
         </is>
       </c>
     </row>
@@ -1979,13 +2573,13 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>1</v>
+        <v>6478</v>
       </c>
       <c r="C33" t="n">
-        <v>13547</v>
+        <v>196</v>
       </c>
       <c r="D33" t="n">
-        <v>733</v>
+        <v>13750</v>
       </c>
     </row>
     <row r="34">
@@ -1995,13 +2589,13 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>2</v>
+        <v>5883</v>
       </c>
       <c r="C34" t="n">
-        <v>6050</v>
+        <v>148</v>
       </c>
       <c r="D34" t="n">
-        <v>0</v>
+        <v>12012</v>
       </c>
     </row>
     <row r="36">
@@ -2033,13 +2627,13 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>0</v>
+        <v>31.7</v>
       </c>
       <c r="C37" t="n">
-        <v>94.90000000000001</v>
+        <v>1</v>
       </c>
       <c r="D37" t="n">
-        <v>5.1</v>
+        <v>67.3</v>
       </c>
     </row>
     <row r="38">
@@ -2049,19 +2643,19 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>0</v>
+        <v>28.8</v>
       </c>
       <c r="C38" t="n">
-        <v>42.4</v>
+        <v>0.7</v>
       </c>
       <c r="D38" t="n">
-        <v>0</v>
+        <v>58.8</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Day 5 — Active seconds: 15776</t>
+          <t>Day 5 — Active seconds: 19332</t>
         </is>
       </c>
     </row>
@@ -2094,13 +2688,13 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>4</v>
+        <v>2782</v>
       </c>
       <c r="C43" t="n">
-        <v>15344</v>
+        <v>95</v>
       </c>
       <c r="D43" t="n">
-        <v>428</v>
+        <v>16455</v>
       </c>
     </row>
     <row r="44">
@@ -2110,13 +2704,13 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>0</v>
+        <v>2267</v>
       </c>
       <c r="C44" t="n">
-        <v>5059</v>
+        <v>49</v>
       </c>
       <c r="D44" t="n">
-        <v>0</v>
+        <v>14249</v>
       </c>
     </row>
     <row r="46">
@@ -2148,13 +2742,13 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>0</v>
+        <v>14.4</v>
       </c>
       <c r="C47" t="n">
-        <v>97.3</v>
+        <v>0.5</v>
       </c>
       <c r="D47" t="n">
-        <v>2.7</v>
+        <v>85.09999999999999</v>
       </c>
     </row>
     <row r="48">
@@ -2164,13 +2758,13 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>0</v>
+        <v>11.7</v>
       </c>
       <c r="C48" t="n">
-        <v>32.1</v>
+        <v>0.3</v>
       </c>
       <c r="D48" t="n">
-        <v>0</v>
+        <v>73.7</v>
       </c>
     </row>
   </sheetData>
@@ -2190,7 +2784,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Day 1 — Active seconds: 18260</t>
+          <t>Day 1 — Active seconds: 19278</t>
         </is>
       </c>
     </row>
@@ -2223,13 +2817,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>9616</v>
+        <v>9508</v>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>190</v>
       </c>
       <c r="D3" t="n">
-        <v>8644</v>
+        <v>9580</v>
       </c>
     </row>
     <row r="4">
@@ -2239,13 +2833,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>8178</v>
+        <v>7956</v>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>171</v>
       </c>
       <c r="D4" t="n">
-        <v>6371</v>
+        <v>8515</v>
       </c>
     </row>
     <row r="6">
@@ -2277,13 +2871,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>52.7</v>
+        <v>49.3</v>
       </c>
       <c r="C7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D7" t="n">
-        <v>47.3</v>
+        <v>49.7</v>
       </c>
     </row>
     <row r="8">
@@ -2293,19 +2887,19 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>44.8</v>
+        <v>41.3</v>
       </c>
       <c r="C8" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="D8" t="n">
-        <v>34.9</v>
+        <v>44.2</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Day 2 — Active seconds: 19929</t>
+          <t>Day 2 — Active seconds: 22130</t>
         </is>
       </c>
     </row>
@@ -2338,13 +2932,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>7948</v>
+        <v>7345</v>
       </c>
       <c r="C13" t="n">
-        <v>0</v>
+        <v>165</v>
       </c>
       <c r="D13" t="n">
-        <v>11981</v>
+        <v>14620</v>
       </c>
     </row>
     <row r="14">
@@ -2354,13 +2948,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>6605</v>
+        <v>6776</v>
       </c>
       <c r="C14" t="n">
-        <v>0</v>
+        <v>125</v>
       </c>
       <c r="D14" t="n">
-        <v>9663</v>
+        <v>14289</v>
       </c>
     </row>
     <row r="16">
@@ -2392,13 +2986,13 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>39.9</v>
+        <v>33.2</v>
       </c>
       <c r="C17" t="n">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="D17" t="n">
-        <v>60.1</v>
+        <v>66.09999999999999</v>
       </c>
     </row>
     <row r="18">
@@ -2408,19 +3002,19 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>33.1</v>
+        <v>30.6</v>
       </c>
       <c r="C18" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="D18" t="n">
-        <v>48.5</v>
+        <v>64.59999999999999</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Day 3 — Active seconds: 18649</t>
+          <t>Day 3 — Active seconds: 21289</t>
         </is>
       </c>
     </row>
@@ -2453,13 +3047,13 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>8094</v>
+        <v>6984</v>
       </c>
       <c r="C23" t="n">
-        <v>0</v>
+        <v>209</v>
       </c>
       <c r="D23" t="n">
-        <v>10555</v>
+        <v>14096</v>
       </c>
     </row>
     <row r="24">
@@ -2469,13 +3063,13 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>5785</v>
+        <v>6043</v>
       </c>
       <c r="C24" t="n">
-        <v>0</v>
+        <v>135</v>
       </c>
       <c r="D24" t="n">
-        <v>7263</v>
+        <v>13697</v>
       </c>
     </row>
     <row r="26">
@@ -2507,13 +3101,13 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>43.4</v>
+        <v>32.8</v>
       </c>
       <c r="C27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D27" t="n">
-        <v>56.6</v>
+        <v>66.2</v>
       </c>
     </row>
     <row r="28">
@@ -2523,19 +3117,19 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>31</v>
+        <v>28.4</v>
       </c>
       <c r="C28" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="D28" t="n">
-        <v>38.9</v>
+        <v>64.3</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Day 4 — Active seconds: 19816</t>
+          <t>Day 4 — Active seconds: 21991</t>
         </is>
       </c>
     </row>
@@ -2568,13 +3162,13 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>7636</v>
+        <v>7124</v>
       </c>
       <c r="C33" t="n">
-        <v>0</v>
+        <v>130</v>
       </c>
       <c r="D33" t="n">
-        <v>12180</v>
+        <v>14737</v>
       </c>
     </row>
     <row r="34">
@@ -2584,13 +3178,13 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>6699</v>
+        <v>6453</v>
       </c>
       <c r="C34" t="n">
-        <v>0</v>
+        <v>181</v>
       </c>
       <c r="D34" t="n">
-        <v>9843</v>
+        <v>14305</v>
       </c>
     </row>
     <row r="36">
@@ -2622,13 +3216,13 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>38.5</v>
+        <v>32.4</v>
       </c>
       <c r="C37" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="D37" t="n">
-        <v>61.5</v>
+        <v>67</v>
       </c>
     </row>
     <row r="38">
@@ -2638,19 +3232,19 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>33.8</v>
+        <v>29.3</v>
       </c>
       <c r="C38" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="D38" t="n">
-        <v>49.7</v>
+        <v>65</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Day 5 — Active seconds: 19805</t>
+          <t>Day 5 — Active seconds: 21831</t>
         </is>
       </c>
     </row>
@@ -2683,13 +3277,13 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>10296</v>
+        <v>3541</v>
       </c>
       <c r="C43" t="n">
-        <v>0</v>
+        <v>79</v>
       </c>
       <c r="D43" t="n">
-        <v>9509</v>
+        <v>18211</v>
       </c>
     </row>
     <row r="44">
@@ -2699,13 +3293,13 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>8665</v>
+        <v>2893</v>
       </c>
       <c r="C44" t="n">
-        <v>0</v>
+        <v>63</v>
       </c>
       <c r="D44" t="n">
-        <v>7836</v>
+        <v>17811</v>
       </c>
     </row>
     <row r="46">
@@ -2737,13 +3331,13 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>52</v>
+        <v>16.2</v>
       </c>
       <c r="C47" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="D47" t="n">
-        <v>48</v>
+        <v>83.40000000000001</v>
       </c>
     </row>
     <row r="48">
@@ -2753,13 +3347,13 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>43.8</v>
+        <v>13.3</v>
       </c>
       <c r="C48" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="D48" t="n">
-        <v>39.6</v>
+        <v>81.59999999999999</v>
       </c>
     </row>
   </sheetData>
@@ -2779,7 +3373,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Day 1 — Active seconds: 13909</t>
+          <t>Day 1 — Active seconds: 14630</t>
         </is>
       </c>
     </row>
@@ -2812,13 +3406,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>580</v>
+        <v>14</v>
       </c>
       <c r="C3" t="n">
-        <v>11592</v>
+        <v>13654</v>
       </c>
       <c r="D3" t="n">
-        <v>1737</v>
+        <v>962</v>
       </c>
     </row>
     <row r="4">
@@ -2828,13 +3422,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>334</v>
+        <v>3</v>
       </c>
       <c r="C4" t="n">
-        <v>7433</v>
+        <v>4516</v>
       </c>
       <c r="D4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -2866,13 +3460,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>4.2</v>
+        <v>0.1</v>
       </c>
       <c r="C7" t="n">
-        <v>83.3</v>
+        <v>93.3</v>
       </c>
       <c r="D7" t="n">
-        <v>12.5</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="8">
@@ -2882,10 +3476,10 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2.4</v>
+        <v>0</v>
       </c>
       <c r="C8" t="n">
-        <v>53.4</v>
+        <v>30.9</v>
       </c>
       <c r="D8" t="n">
         <v>0</v>
@@ -2894,7 +3488,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Day 2 — Active seconds: 13371</t>
+          <t>Day 2 — Active seconds: 16319</t>
         </is>
       </c>
     </row>
@@ -2927,13 +3521,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>144</v>
+        <v>5</v>
       </c>
       <c r="C13" t="n">
-        <v>12098</v>
+        <v>15814</v>
       </c>
       <c r="D13" t="n">
-        <v>1129</v>
+        <v>500</v>
       </c>
     </row>
     <row r="14">
@@ -2943,10 +3537,599 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>82</v>
+        <v>4</v>
       </c>
       <c r="C14" t="n">
-        <v>9126</v>
+        <v>8940</v>
+      </c>
+      <c r="D14" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Percentages (%)</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Inside NBBO</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>At NBBO</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Outside NBBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" t="n">
+        <v>96.90000000000001</v>
+      </c>
+      <c r="D17" t="n">
+        <v>3.1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" t="n">
+        <v>54.8</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Day 3 — Active seconds: 16080</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Counts</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Inside NBBO</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>At NBBO</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Outside NBBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>10</v>
+      </c>
+      <c r="C23" t="n">
+        <v>15309</v>
+      </c>
+      <c r="D23" t="n">
+        <v>761</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>11</v>
+      </c>
+      <c r="C24" t="n">
+        <v>7981</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Percentages (%)</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Inside NBBO</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>At NBBO</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Outside NBBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C27" t="n">
+        <v>95.2</v>
+      </c>
+      <c r="D27" t="n">
+        <v>4.7</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C28" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="D28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Day 4 — Active seconds: 16366</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Counts</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Inside NBBO</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>At NBBO</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Outside NBBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>6</v>
+      </c>
+      <c r="C33" t="n">
+        <v>15588</v>
+      </c>
+      <c r="D33" t="n">
+        <v>772</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>6</v>
+      </c>
+      <c r="C34" t="n">
+        <v>8763</v>
+      </c>
+      <c r="D34" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Percentages (%)</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Inside NBBO</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>At NBBO</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Outside NBBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" t="n">
+        <v>95.2</v>
+      </c>
+      <c r="D37" t="n">
+        <v>4.7</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" t="n">
+        <v>53.5</v>
+      </c>
+      <c r="D38" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Day 5 — Active seconds: 17317</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Counts</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Inside NBBO</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>At NBBO</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Outside NBBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>1</v>
+      </c>
+      <c r="C43" t="n">
+        <v>16875</v>
+      </c>
+      <c r="D43" t="n">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" t="n">
+        <v>7480</v>
+      </c>
+      <c r="D44" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Percentages (%)</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Inside NBBO</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>At NBBO</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Outside NBBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" t="n">
+        <v>97.40000000000001</v>
+      </c>
+      <c r="D47" t="n">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" t="n">
+        <v>43.2</v>
+      </c>
+      <c r="D48" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D48"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Day 1 — Active seconds: 16815</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Counts</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Inside NBBO</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>At NBBO</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Outside NBBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>35</v>
+      </c>
+      <c r="C3" t="n">
+        <v>15817</v>
+      </c>
+      <c r="D3" t="n">
+        <v>963</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>5</v>
+      </c>
+      <c r="C4" t="n">
+        <v>10598</v>
+      </c>
+      <c r="D4" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Percentages (%)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Inside NBBO</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>At NBBO</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Outside NBBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C7" t="n">
+        <v>94.09999999999999</v>
+      </c>
+      <c r="D7" t="n">
+        <v>5.7</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" t="n">
+        <v>63</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Day 2 — Active seconds: 19269</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Counts</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Inside NBBO</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>At NBBO</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Outside NBBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>9</v>
+      </c>
+      <c r="C13" t="n">
+        <v>18714</v>
+      </c>
+      <c r="D13" t="n">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>7</v>
+      </c>
+      <c r="C14" t="n">
+        <v>16294</v>
       </c>
       <c r="D14" t="n">
         <v>5</v>
@@ -2981,13 +4164,13 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>1.1</v>
+        <v>0</v>
       </c>
       <c r="C17" t="n">
-        <v>90.5</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="D17" t="n">
-        <v>8.4</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="18">
@@ -2997,10 +4180,10 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="C18" t="n">
-        <v>68.3</v>
+        <v>84.59999999999999</v>
       </c>
       <c r="D18" t="n">
         <v>0</v>
@@ -3009,7 +4192,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Day 3 — Active seconds: 15014</t>
+          <t>Day 3 — Active seconds: 19440</t>
         </is>
       </c>
     </row>
@@ -3042,13 +4225,13 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>490</v>
+        <v>22</v>
       </c>
       <c r="C23" t="n">
-        <v>13273</v>
+        <v>18615</v>
       </c>
       <c r="D23" t="n">
-        <v>1251</v>
+        <v>803</v>
       </c>
     </row>
     <row r="24">
@@ -3058,13 +4241,13 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>346</v>
+        <v>16</v>
       </c>
       <c r="C24" t="n">
-        <v>9501</v>
+        <v>15745</v>
       </c>
       <c r="D24" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="26">
@@ -3096,13 +4279,13 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>3.3</v>
+        <v>0.1</v>
       </c>
       <c r="C27" t="n">
-        <v>88.40000000000001</v>
+        <v>95.8</v>
       </c>
       <c r="D27" t="n">
-        <v>8.300000000000001</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="28">
@@ -3112,10 +4295,10 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>2.3</v>
+        <v>0.1</v>
       </c>
       <c r="C28" t="n">
-        <v>63.3</v>
+        <v>81</v>
       </c>
       <c r="D28" t="n">
         <v>0</v>
@@ -3124,7 +4307,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Day 4 — Active seconds: 16393</t>
+          <t>Day 4 — Active seconds: 19294</t>
         </is>
       </c>
     </row>
@@ -3157,13 +4340,13 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>429</v>
+        <v>15</v>
       </c>
       <c r="C33" t="n">
-        <v>14964</v>
+        <v>18489</v>
       </c>
       <c r="D33" t="n">
-        <v>1000</v>
+        <v>790</v>
       </c>
     </row>
     <row r="34">
@@ -3173,13 +4356,13 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>265</v>
+        <v>17</v>
       </c>
       <c r="C34" t="n">
-        <v>10592</v>
+        <v>16128</v>
       </c>
       <c r="D34" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="36">
@@ -3211,13 +4394,13 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>2.6</v>
+        <v>0.1</v>
       </c>
       <c r="C37" t="n">
-        <v>91.3</v>
+        <v>95.8</v>
       </c>
       <c r="D37" t="n">
-        <v>6.1</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="38">
@@ -3227,10 +4410,10 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>1.6</v>
+        <v>0.1</v>
       </c>
       <c r="C38" t="n">
-        <v>64.59999999999999</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="D38" t="n">
         <v>0</v>
@@ -3239,7 +4422,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Day 5 — Active seconds: 16456</t>
+          <t>Day 5 — Active seconds: 20491</t>
         </is>
       </c>
     </row>
@@ -3272,13 +4455,13 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>427</v>
+        <v>13</v>
       </c>
       <c r="C43" t="n">
-        <v>14729</v>
+        <v>19991</v>
       </c>
       <c r="D43" t="n">
-        <v>1300</v>
+        <v>487</v>
       </c>
     </row>
     <row r="44">
@@ -3288,13 +4471,13 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>265</v>
+        <v>1</v>
       </c>
       <c r="C44" t="n">
-        <v>9966</v>
+        <v>16133</v>
       </c>
       <c r="D44" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="46">
@@ -3326,13 +4509,13 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>2.6</v>
+        <v>0.1</v>
       </c>
       <c r="C47" t="n">
-        <v>89.5</v>
+        <v>97.59999999999999</v>
       </c>
       <c r="D47" t="n">
-        <v>7.9</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="48">
@@ -3342,13 +4525,1780 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>1.6</v>
+        <v>0</v>
       </c>
       <c r="C48" t="n">
-        <v>60.6</v>
+        <v>78.7</v>
       </c>
       <c r="D48" t="n">
         <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D48"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Day 1 — Active seconds: 20307</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Counts</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Inside NBBO</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>At NBBO</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Outside NBBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>11323</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" t="n">
+        <v>8984</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>10669</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" t="n">
+        <v>7450</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Percentages (%)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Inside NBBO</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>At NBBO</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Outside NBBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>55.8</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" t="n">
+        <v>44.2</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>52.5</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" t="n">
+        <v>36.7</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Day 2 — Active seconds: 21206</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Counts</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Inside NBBO</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>At NBBO</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Outside NBBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>8829</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" t="n">
+        <v>12377</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>8158</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" t="n">
+        <v>11009</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Percentages (%)</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Inside NBBO</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>At NBBO</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Outside NBBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>41.6</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" t="n">
+        <v>58.4</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" t="n">
+        <v>51.9</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Day 3 — Active seconds: 20249</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Counts</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Inside NBBO</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>At NBBO</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Outside NBBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>9370</v>
+      </c>
+      <c r="C23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" t="n">
+        <v>10879</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>8662</v>
+      </c>
+      <c r="C24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" t="n">
+        <v>9094</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Percentages (%)</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Inside NBBO</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>At NBBO</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Outside NBBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>46.3</v>
+      </c>
+      <c r="C27" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" t="n">
+        <v>53.7</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>42.8</v>
+      </c>
+      <c r="C28" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" t="n">
+        <v>44.9</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Day 4 — Active seconds: 20938</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Counts</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Inside NBBO</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>At NBBO</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Outside NBBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>8409</v>
+      </c>
+      <c r="C33" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" t="n">
+        <v>12529</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>7961</v>
+      </c>
+      <c r="C34" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" t="n">
+        <v>10872</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Percentages (%)</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Inside NBBO</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>At NBBO</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Outside NBBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>40.2</v>
+      </c>
+      <c r="C37" t="n">
+        <v>0</v>
+      </c>
+      <c r="D37" t="n">
+        <v>59.8</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>38</v>
+      </c>
+      <c r="C38" t="n">
+        <v>0</v>
+      </c>
+      <c r="D38" t="n">
+        <v>51.9</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Day 5 — Active seconds: 21295</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Counts</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Inside NBBO</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>At NBBO</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Outside NBBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>11403</v>
+      </c>
+      <c r="C43" t="n">
+        <v>0</v>
+      </c>
+      <c r="D43" t="n">
+        <v>9892</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>10625</v>
+      </c>
+      <c r="C44" t="n">
+        <v>0</v>
+      </c>
+      <c r="D44" t="n">
+        <v>8821</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Percentages (%)</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Inside NBBO</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>At NBBO</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Outside NBBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>53.5</v>
+      </c>
+      <c r="C47" t="n">
+        <v>0</v>
+      </c>
+      <c r="D47" t="n">
+        <v>46.5</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>49.9</v>
+      </c>
+      <c r="C48" t="n">
+        <v>0</v>
+      </c>
+      <c r="D48" t="n">
+        <v>41.4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D48"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Day 1 — Active seconds: 21077</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Counts</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Inside NBBO</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>At NBBO</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Outside NBBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>11837</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" t="n">
+        <v>9240</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>11277</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" t="n">
+        <v>8130</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Percentages (%)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Inside NBBO</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>At NBBO</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Outside NBBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>56.2</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" t="n">
+        <v>43.8</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>53.5</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" t="n">
+        <v>38.6</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Day 2 — Active seconds: 21893</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Counts</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Inside NBBO</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>At NBBO</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Outside NBBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>9230</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" t="n">
+        <v>12663</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>8635</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" t="n">
+        <v>11790</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Percentages (%)</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Inside NBBO</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>At NBBO</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Outside NBBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>42.2</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" t="n">
+        <v>57.8</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>39.4</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" t="n">
+        <v>53.9</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Day 3 — Active seconds: 21132</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Counts</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Inside NBBO</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>At NBBO</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Outside NBBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>9915</v>
+      </c>
+      <c r="C23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" t="n">
+        <v>11217</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>9322</v>
+      </c>
+      <c r="C24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" t="n">
+        <v>10008</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Percentages (%)</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Inside NBBO</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>At NBBO</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Outside NBBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>46.9</v>
+      </c>
+      <c r="C27" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" t="n">
+        <v>53.1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>44.1</v>
+      </c>
+      <c r="C28" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" t="n">
+        <v>47.4</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Day 4 — Active seconds: 21868</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Counts</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Inside NBBO</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>At NBBO</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Outside NBBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>8960</v>
+      </c>
+      <c r="C33" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" t="n">
+        <v>12908</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>8554</v>
+      </c>
+      <c r="C34" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" t="n">
+        <v>11924</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Percentages (%)</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Inside NBBO</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>At NBBO</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Outside NBBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>41</v>
+      </c>
+      <c r="C37" t="n">
+        <v>0</v>
+      </c>
+      <c r="D37" t="n">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>39.1</v>
+      </c>
+      <c r="C38" t="n">
+        <v>0</v>
+      </c>
+      <c r="D38" t="n">
+        <v>54.5</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Day 5 — Active seconds: 21834</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Counts</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Inside NBBO</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>At NBBO</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Outside NBBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>11701</v>
+      </c>
+      <c r="C43" t="n">
+        <v>0</v>
+      </c>
+      <c r="D43" t="n">
+        <v>10133</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>10899</v>
+      </c>
+      <c r="C44" t="n">
+        <v>0</v>
+      </c>
+      <c r="D44" t="n">
+        <v>9507</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Percentages (%)</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Inside NBBO</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>At NBBO</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Outside NBBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>53.6</v>
+      </c>
+      <c r="C47" t="n">
+        <v>0</v>
+      </c>
+      <c r="D47" t="n">
+        <v>46.4</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>49.9</v>
+      </c>
+      <c r="C48" t="n">
+        <v>0</v>
+      </c>
+      <c r="D48" t="n">
+        <v>43.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D48"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Day 1 — Active seconds: 15082</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Counts</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Inside NBBO</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>At NBBO</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Outside NBBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>648</v>
+      </c>
+      <c r="C3" t="n">
+        <v>12660</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1774</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>463</v>
+      </c>
+      <c r="C4" t="n">
+        <v>8763</v>
+      </c>
+      <c r="D4" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Percentages (%)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Inside NBBO</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>At NBBO</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Outside NBBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="C7" t="n">
+        <v>83.90000000000001</v>
+      </c>
+      <c r="D7" t="n">
+        <v>11.8</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="C8" t="n">
+        <v>58.1</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Day 2 — Active seconds: 14021</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Counts</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Inside NBBO</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>At NBBO</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Outside NBBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>147</v>
+      </c>
+      <c r="C13" t="n">
+        <v>12631</v>
+      </c>
+      <c r="D13" t="n">
+        <v>1243</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>114</v>
+      </c>
+      <c r="C14" t="n">
+        <v>9964</v>
+      </c>
+      <c r="D14" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Percentages (%)</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Inside NBBO</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>At NBBO</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Outside NBBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>1</v>
+      </c>
+      <c r="C17" t="n">
+        <v>90.09999999999999</v>
+      </c>
+      <c r="D17" t="n">
+        <v>8.9</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="C18" t="n">
+        <v>71.09999999999999</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Day 3 — Active seconds: 15847</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Counts</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Inside NBBO</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>At NBBO</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Outside NBBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>564</v>
+      </c>
+      <c r="C23" t="n">
+        <v>13952</v>
+      </c>
+      <c r="D23" t="n">
+        <v>1331</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>436</v>
+      </c>
+      <c r="C24" t="n">
+        <v>10650</v>
+      </c>
+      <c r="D24" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Percentages (%)</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Inside NBBO</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>At NBBO</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Outside NBBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="C27" t="n">
+        <v>88</v>
+      </c>
+      <c r="D27" t="n">
+        <v>8.4</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="C28" t="n">
+        <v>67.2</v>
+      </c>
+      <c r="D28" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Day 4 — Active seconds: 17780</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Counts</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Inside NBBO</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>At NBBO</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Outside NBBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>478</v>
+      </c>
+      <c r="C33" t="n">
+        <v>16208</v>
+      </c>
+      <c r="D33" t="n">
+        <v>1094</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>318</v>
+      </c>
+      <c r="C34" t="n">
+        <v>12447</v>
+      </c>
+      <c r="D34" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Percentages (%)</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Inside NBBO</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>At NBBO</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Outside NBBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="C37" t="n">
+        <v>91.2</v>
+      </c>
+      <c r="D37" t="n">
+        <v>6.2</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="C38" t="n">
+        <v>70</v>
+      </c>
+      <c r="D38" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Day 5 — Active seconds: 17755</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Counts</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Inside NBBO</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>At NBBO</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Outside NBBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>487</v>
+      </c>
+      <c r="C43" t="n">
+        <v>15979</v>
+      </c>
+      <c r="D43" t="n">
+        <v>1289</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>352</v>
+      </c>
+      <c r="C44" t="n">
+        <v>11888</v>
+      </c>
+      <c r="D44" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Percentages (%)</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Inside NBBO</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>At NBBO</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Outside NBBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Bid</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="C47" t="n">
+        <v>90</v>
+      </c>
+      <c r="D47" t="n">
+        <v>7.3</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Ask</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>2</v>
+      </c>
+      <c r="C48" t="n">
+        <v>67</v>
+      </c>
+      <c r="D48" t="n">
+        <v>0.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>